<commit_message>
S06 dataset: remover fuga do gabarito + limpar anomalias acidentais
- apagada a folha oculta _NotasInternas (gabarito completo, distribuido
  aos formandos) e removido "(anomalia:...)" do Objecto da linha 6
- 4 contratos com compromisso>adjudicado acidental corrigidos (subido o
  Valor Adjudicado); ficam as 3 anomalias plantadas
- taxa de execucao inalterada (Acad 61 / Fin 75 / RH 70 / DSI 79; global 72)

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sessoes/sessao-06/Dataset_S06_Execucao_Orcamental.xlsx
+++ b/sessoes/sessao-06/Dataset_S06_Execucao_Orcamental.xlsx
@@ -10,7 +10,6 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contratos" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Anomalias detectadas" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Indicadores" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_NotasInternas" sheetId="4" state="hidden" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -641,7 +640,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Serviços de auditoria externa (anomalia: pagamento &gt; compromisso)</t>
+          <t>Serviços de auditoria externa</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -709,7 +708,7 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>175776.57</v>
+        <v>183355.86</v>
       </c>
       <c r="G7" t="n">
         <v>181239.21</v>
@@ -1481,7 +1480,7 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>18710.52</v>
+        <v>19665.91</v>
       </c>
       <c r="G22" t="n">
         <v>19574.78</v>
@@ -1591,7 +1590,7 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>177850.91</v>
+        <v>183549.08</v>
       </c>
       <c r="G24" t="n">
         <v>179548.54</v>
@@ -2203,7 +2202,7 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>96162.10000000001</v>
+        <v>99567.64</v>
       </c>
       <c r="G35" t="n">
         <v>97187.13</v>
@@ -2697,119 +2696,4 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A15"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="9" t="inlineStr">
-        <is>
-          <t>NOTAS INTERNAS — não distribuir aos formandos</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Este ficheiro tem 'sujidade calibrada' para o exercício da Sessão 6.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>1. Datas em 3 formatos mistos (DD/MM/YYYY, DD-MM-YYYY, DD MMM YYYY).</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2. Valores monetários ocasionalmente como string com '€' ou '€ '.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>3. N.º contratos com formatos inconsistentes (com/sem espaços, sublinhado, etc.).</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>4. Adjudicatários com grafias variadas (mesma empresa, diferentes maiúsculas/abreviações).</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>5. Linha de subtotal MESCLADA no meio dos dados (linha ~17) — confunde o Copilot.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>6. Linha de TOTAL final com valor deliberadamente mal calculado.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>7. 3 anomalias legais embebidas:</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   - Contrato com pagamento &gt; compromisso (auditoria externa)</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   - Contrato sem cabimento (aquisição equipamento rede urgente)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   - Contrato com compromisso &gt; valor adjudicado (limpeza)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Os formandos detectarão estas anomalias na Sub-A (exercício guiado).</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Devem propor reformulação dos dados na fase de 'preparação para análise'.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>